<commit_message>
working , fpga issues at rs422 pins
</commit_message>
<xml_diff>
--- a/PMSS FPGA pin Mapping Input/PMSS PRO FPGA IO Signal mapping.xlsx
+++ b/PMSS FPGA pin Mapping Input/PMSS PRO FPGA IO Signal mapping.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12300" firstSheet="1" activeTab="1"/>
+    <workbookView windowWidth="14400" windowHeight="12180" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="4" r:id="rId1"/>
@@ -4692,6 +4692,9 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A2:D147" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600"/>
   <headerFooter>

</xml_diff>